<commit_message>
include childrens Endpoint in ERF
</commit_message>
<xml_diff>
--- a/data/ETCHE/functionsETCHE.xlsx
+++ b/data/ETCHE/functionsETCHE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dokumente_lokal\LÄRM Projekte\Quantifizierung von Lärmschadenskosten\GitHub Repository\Hessen_END_Healthiar\data\ETCHE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lochmannm\Documents\GitHub\END2DALY\data\ETCHE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF8484D3-AB46-45B6-BAEC-CC15FA2AC982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A800516-53D4-4F8D-8997-F2F359AD34B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{48A8F245-2396-4F0B-B734-4CFAEB6227B4}"/>
+    <workbookView xWindow="28680" yWindow="-4140" windowWidth="29040" windowHeight="15720" xr2:uid="{48A8F245-2396-4F0B-B734-4CFAEB6227B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="68">
   <si>
     <t>Guski et al. (2017)</t>
   </si>
@@ -215,6 +215,33 @@
   </si>
   <si>
     <t>für END_model fehlt IHD</t>
+  </si>
+  <si>
+    <t>ETCHE23_model</t>
+  </si>
+  <si>
+    <t>ETCHE24_model</t>
+  </si>
+  <si>
+    <t>Behavioural problems</t>
+  </si>
+  <si>
+    <t>Overweight</t>
+  </si>
+  <si>
+    <t>ifelse(c&gt;threshold,(c-threshold)*1.073,0)</t>
+  </si>
+  <si>
+    <t>ifelse(c&gt;threshold,(c-threshold)*1.063,0)</t>
+  </si>
+  <si>
+    <t>Engelmann ETC HE Report 2024/11, ch 3.3.2</t>
+  </si>
+  <si>
+    <t>Engelmann ETC HE Report 2024/11</t>
+  </si>
+  <si>
+    <t>Engelmann ETC HE Report 2024/11, ch 3.3.5</t>
   </si>
 </sst>
 </file>
@@ -274,14 +301,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>349250</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>153755</xdr:colOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>77555</xdr:colOff>
       <xdr:row>50</xdr:row>
       <xdr:rowOff>83846</xdr:rowOff>
     </xdr:to>
@@ -306,8 +333,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8731250" y="0"/>
-          <a:ext cx="9710505" cy="9135771"/>
+          <a:off x="18830925" y="0"/>
+          <a:ext cx="9707330" cy="9132596"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -318,16 +345,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>704272</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>23091</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>416095</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>93501</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>4162802</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>65624</xdr:rowOff>
+      <xdr:colOff>2254628</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>123333</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -350,8 +377,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1466272" y="4271818"/>
-          <a:ext cx="6839905" cy="2810267"/>
+          <a:off x="416095" y="4934442"/>
+          <a:ext cx="6993239" cy="2725594"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -363,15 +390,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:colOff>391832</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>173692</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>2464824</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>133482</xdr:rowOff>
+      <xdr:colOff>2812206</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>26279</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -394,12 +421,73 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="47625" y="7153275"/>
-          <a:ext cx="7335274" cy="943107"/>
+          <a:off x="391832" y="7524751"/>
+          <a:ext cx="7575080" cy="934702"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3650961</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>141720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>30694</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>31462</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Grafik 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4C9C822-88BB-25CF-DAA5-67684AA255AB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8811779" y="5337175"/>
+          <a:ext cx="6756499" cy="2837007"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -704,22 +792,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8156CAC4-1F63-4625-9494-276B4F46068B}">
-  <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="77.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="37.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="77.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="37.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -753,8 +841,14 @@
       <c r="K1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>59</v>
+      </c>
+      <c r="M1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -788,8 +882,14 @@
       <c r="K2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -823,8 +923,14 @@
       <c r="K3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -858,8 +964,14 @@
       <c r="K4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -893,8 +1005,14 @@
       <c r="K5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -928,8 +1046,14 @@
       <c r="K6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -963,8 +1087,14 @@
       <c r="K7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -998,8 +1128,14 @@
       <c r="K8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1033,8 +1169,14 @@
       <c r="K9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -1065,8 +1207,14 @@
       <c r="K10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -1097,8 +1245,14 @@
       <c r="K11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -1129,8 +1283,14 @@
       <c r="K12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1161,8 +1321,14 @@
       <c r="K13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1193,8 +1359,14 @@
       <c r="K14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1225,8 +1397,14 @@
       <c r="K15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -1257,8 +1435,14 @@
       <c r="K16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -1289,8 +1473,14 @@
       <c r="K17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -1321,8 +1511,14 @@
       <c r="K18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -1355,6 +1551,316 @@
       </c>
       <c r="K19">
         <v>0</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F20" t="s">
+        <v>47</v>
+      </c>
+      <c r="G20" t="s">
+        <v>3</v>
+      </c>
+      <c r="H20">
+        <v>50</v>
+      </c>
+      <c r="I20" t="s">
+        <v>66</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" t="s">
+        <v>5</v>
+      </c>
+      <c r="F21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G21" t="s">
+        <v>3</v>
+      </c>
+      <c r="H21">
+        <v>50</v>
+      </c>
+      <c r="I21" t="s">
+        <v>66</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" t="s">
+        <v>5</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G22" t="s">
+        <v>3</v>
+      </c>
+      <c r="H22">
+        <v>45</v>
+      </c>
+      <c r="I22" t="s">
+        <v>65</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" t="s">
+        <v>6</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G23" t="s">
+        <v>3</v>
+      </c>
+      <c r="H23">
+        <v>45</v>
+      </c>
+      <c r="I23" t="s">
+        <v>65</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" t="s">
+        <v>29</v>
+      </c>
+      <c r="E24" t="s">
+        <v>7</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G24" t="s">
+        <v>3</v>
+      </c>
+      <c r="H24">
+        <v>45</v>
+      </c>
+      <c r="I24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25" t="s">
+        <v>5</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G25" t="s">
+        <v>3</v>
+      </c>
+      <c r="H25">
+        <v>45</v>
+      </c>
+      <c r="I25" t="s">
+        <v>67</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" t="s">
+        <v>6</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G26" t="s">
+        <v>3</v>
+      </c>
+      <c r="H26">
+        <v>45</v>
+      </c>
+      <c r="I26" t="s">
+        <v>67</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" t="s">
+        <v>27</v>
+      </c>
+      <c r="D27" t="s">
+        <v>29</v>
+      </c>
+      <c r="E27" t="s">
+        <v>7</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G27" t="s">
+        <v>3</v>
+      </c>
+      <c r="H27">
+        <v>45</v>
+      </c>
+      <c r="I27" t="s">
+        <v>67</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1366,14 +1872,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1566883E-42F0-44A5-A5A7-BA00A033D6E6}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>55</v>
       </c>
@@ -1381,7 +1887,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>51</v>
       </c>
@@ -1389,7 +1895,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>51</v>
       </c>
@@ -1397,12 +1903,12 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
workaround different handling of RR and AR
</commit_message>
<xml_diff>
--- a/data/ETCHE/functionsETCHE.xlsx
+++ b/data/ETCHE/functionsETCHE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lochmannm\Documents\GitHub\END2DALY\data\ETCHE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C65F40B-D845-4720-9A07-F6E3AE218AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2262A98E-BA7F-4C98-BC97-BFE65101BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1980" windowWidth="29040" windowHeight="17520" xr2:uid="{48A8F245-2396-4F0B-B734-4CFAEB6227B4}"/>
   </bookViews>
@@ -202,6 +202,30 @@
     <t>Engelmann ETC HE Report 2024/11, ch 3.3.5</t>
   </si>
   <si>
+    <t>ifelse (c &gt;= threshold, 1 / (1 + exp(-(log(0.1 / 0.9) + (log(1.38) / 10 * (c - 50))))), 0.1)</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>(78.9270 - 3.1162 * c + 0.0342 * c^2)/100</t>
+  </si>
+  <si>
+    <t>(38.1596 - 2.05538 * c + 0.0285 * c^2)/100</t>
+  </si>
+  <si>
+    <t>(-50.9693 + 1.0168 * c + 0.0072 * c^2)/100</t>
+  </si>
+  <si>
+    <t>(19.4312 - 0.9336 * c + 0.0126 * c^2)/100</t>
+  </si>
+  <si>
+    <t>(67.5406 - 3.1852 * c + 0.0391 * c^2)/100</t>
+  </si>
+  <si>
+    <t>(16.7885 - 0.9293 * c + 0.0198 * c^2)/100</t>
+  </si>
+  <si>
     <t>exp(log(1.055)/10*(c-threshold))</t>
   </si>
   <si>
@@ -215,30 +239,6 @@
   </si>
   <si>
     <t>exp(log(1.063)/10*(c-threshold))</t>
-  </si>
-  <si>
-    <t>ifelse (c &gt;= threshold, 1 / (1 + exp(-(log(0.1 / 0.9) + (log(1.38) / 10 * (c - 50))))), 0.1)</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>(78.9270 - 3.1162 * c + 0.0342 * c^2)/100</t>
-  </si>
-  <si>
-    <t>(38.1596 - 2.05538 * c + 0.0285 * c^2)/100</t>
-  </si>
-  <si>
-    <t>(-50.9693 + 1.0168 * c + 0.0072 * c^2)/100</t>
-  </si>
-  <si>
-    <t>(19.4312 - 0.9336 * c + 0.0126 * c^2)/100</t>
-  </si>
-  <si>
-    <t>(67.5406 - 3.1852 * c + 0.0391 * c^2)/100</t>
-  </si>
-  <si>
-    <t>(16.7885 - 0.9293 * c + 0.0198 * c^2)/100</t>
   </si>
 </sst>
 </file>
@@ -862,7 +862,7 @@
         <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="G2" t="s">
         <v>3</v>
@@ -903,7 +903,7 @@
         <v>6</v>
       </c>
       <c r="F3" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G3" t="s">
         <v>3</v>
@@ -944,7 +944,7 @@
         <v>7</v>
       </c>
       <c r="F4" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="G4" t="s">
         <v>3</v>
@@ -985,7 +985,7 @@
         <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G5" t="s">
         <v>3</v>
@@ -1026,7 +1026,7 @@
         <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -1067,7 +1067,7 @@
         <v>6</v>
       </c>
       <c r="F7" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G7" t="s">
         <v>4</v>
@@ -1108,7 +1108,7 @@
         <v>7</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G8" t="s">
         <v>4</v>
@@ -1149,7 +1149,7 @@
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G9" t="s">
         <v>4</v>
@@ -1190,7 +1190,7 @@
         <v>5</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="G10" t="s">
         <v>3</v>
@@ -1228,7 +1228,7 @@
         <v>6</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="G11" t="s">
         <v>3</v>
@@ -1266,7 +1266,7 @@
         <v>7</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="G12" t="s">
         <v>3</v>
@@ -1304,7 +1304,7 @@
         <v>5</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="G13" t="s">
         <v>3</v>
@@ -1342,7 +1342,7 @@
         <v>6</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="G14" t="s">
         <v>3</v>
@@ -1380,7 +1380,7 @@
         <v>7</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="G15" t="s">
         <v>3</v>
@@ -1418,7 +1418,7 @@
         <v>5</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="G16" t="s">
         <v>3</v>
@@ -1456,7 +1456,7 @@
         <v>6</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="G17" t="s">
         <v>3</v>
@@ -1494,7 +1494,7 @@
         <v>7</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="G18" t="s">
         <v>3</v>
@@ -1532,7 +1532,7 @@
         <v>7</v>
       </c>
       <c r="F19" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G19" t="s">
         <v>3</v>
@@ -1573,7 +1573,7 @@
         <v>6</v>
       </c>
       <c r="F20" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G20" t="s">
         <v>3</v>
@@ -1614,7 +1614,7 @@
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G21" t="s">
         <v>3</v>
@@ -1655,7 +1655,7 @@
         <v>5</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="G22" t="s">
         <v>3</v>
@@ -1693,7 +1693,7 @@
         <v>6</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="G23" t="s">
         <v>3</v>
@@ -1731,7 +1731,7 @@
         <v>7</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="G24" t="s">
         <v>3</v>
@@ -1769,7 +1769,7 @@
         <v>5</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="G25" t="s">
         <v>3</v>
@@ -1807,7 +1807,7 @@
         <v>6</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="G26" t="s">
         <v>3</v>
@@ -1845,7 +1845,7 @@
         <v>7</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="G27" t="s">
         <v>3</v>

</xml_diff>